<commit_message>
fix(export): barcha yangi kiritilgan talabalar eksportlarga to'liq kiritildi va real-vaqtda olinishi ta'minlandi
</commit_message>
<xml_diff>
--- a/hisobotlar/1-kurs_Sorovnoma_Topshirmaganlar_Hisoboti.xlsx
+++ b/hisobotlar/1-kurs_Sorovnoma_Topshirmaganlar_Hisoboti.xlsx
@@ -9,11 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Umumiy tahlil" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Barcha topshirmaganlar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-02" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-03" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-04" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-05" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-06" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-01" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-02" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-03" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-04" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-05" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-06" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guruh 26-07" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -98,17 +100,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -178,35 +180,26 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -215,6 +208,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -673,58 +675,58 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>14</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>0</v>
+          <t>93.3%</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="4" t="n">
-        <v>0</v>
+      <c r="I5" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>26-02</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>Ochilov.D</t>
         </is>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="9" t="n">
         <v>31</v>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>91.2%</t>
         </is>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="G6" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="11" t="n">
+      <c r="I6" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -753,48 +755,48 @@
           <t>73.5%</t>
         </is>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="7" t="n">
         <v>9</v>
       </c>
       <c r="H7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="I7" s="11" t="n">
+      <c r="I7" s="8" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>26-04</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>Xamdamova.M</t>
         </is>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="10" t="n">
         <v>32</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>93.8%</t>
         </is>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="I8" s="7" t="n">
+      <c r="I8" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -823,48 +825,48 @@
           <t>90.6%</t>
         </is>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="I9" s="11" t="n">
+      <c r="I9" s="8" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>26-06</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Yuldashev.O</t>
         </is>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>85.3%</t>
         </is>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G10" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H10" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I10" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -883,7 +885,7 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>0</v>
@@ -893,14 +895,14 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n">
-        <v>0</v>
+      <c r="G11" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="4" t="n">
-        <v>0</v>
+      <c r="I11" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -912,24 +914,24 @@
       </c>
       <c r="C12" s="12" t="inlineStr"/>
       <c r="D12" s="12" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E12" s="12" t="n">
         <v>158</v>
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>87.8%</t>
+          <t>86.8%</t>
         </is>
       </c>
       <c r="G12" s="12" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H12" s="12" t="n">
         <v>16</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -943,7 +945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="79" customWidth="1" min="1" max="1"/>
@@ -960,7 +962,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SO'ROVNOMA TOPSHIRMAGAN BARCHA 1-KURS TALABALARI (22 NAFAR)</t>
+          <t>SO'ROVNOMA TOPSHIRMAGAN BARCHA 1-KURS TALABALARI (24 NAFAR)</t>
         </is>
       </c>
     </row>
@@ -1025,27 +1027,27 @@
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>26-02</t>
+          <t>26-01</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Ochilov.D</t>
+          <t>Mirzayeva.D</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>Nurillayeva Dilsuz Mashrabovna</t>
+          <t>Shermatova Gulsun Xurshid qizi</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>AD4774693</t>
+          <t>AE5836574</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>42506912640010</t>
+          <t>60802085590029</t>
         </is>
       </c>
       <c r="G5" s="14" t="inlineStr">
@@ -1053,7 +1055,7 @@
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
         </is>
@@ -1094,7 +1096,7 @@
           <t>+998 77 833-82-72</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -1135,7 +1137,7 @@
           <t>+998 91 219-20-99</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -1148,78 +1150,78 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
+          <t>26-02</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Ochilov.D</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Nurillayeva Dilsuz Mashrabovna</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>AD4774693</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>42506912640010</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>Mavjud emas</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Telefoni yo'q (aniqlash zarur)</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
           <t>26-03</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>A.Asraliyev</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Aliqulova Shaxzoda Anvar qizi</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>AC1827958</t>
         </is>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>60301037890018</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="17" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>26-03</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>A.Asraliyev</t>
-        </is>
-      </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>Ibragimova Gulnoza Isroil qizi</t>
-        </is>
-      </c>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>AE4115057</t>
-        </is>
-      </c>
-      <c r="F9" s="17" t="inlineStr">
-        <is>
-          <t>60606085680085</t>
-        </is>
-      </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>+998 95 259-06-25 / +998 99 152-33-71 (Otasi / Onasi)</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
@@ -1240,25 +1242,25 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Izzatulloyeva Vazira G'ayratzoda</t>
+          <t>Ibragimova Gulnoza Isroil qizi</t>
         </is>
       </c>
       <c r="E10" s="17" t="inlineStr">
         <is>
-          <t>AE5671026</t>
+          <t>AE4115057</t>
         </is>
       </c>
       <c r="F10" s="17" t="inlineStr">
         <is>
-          <t>42004975680094</t>
+          <t>60606085680085</t>
         </is>
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>+998 87 358-87-97 / +998 88 632-19-72 (Otasi / Onasi)</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
+          <t>+998 95 259-06-25 / +998 99 152-33-71 (Otasi / Onasi)</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -1281,191 +1283,191 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
+          <t>Izzatulloyeva Vazira G'ayratzoda</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>AE5671026</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>42004975680094</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>+998 87 358-87-97 / +998 88 632-19-72 (Otasi / Onasi)</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Telefoni bor (bog'lanish mumkin)</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>26-03</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>A.Asraliyev</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
           <t>Murtazayeva Kamola Jamoliddin qizi</t>
         </is>
       </c>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>AC1458884</t>
         </is>
       </c>
-      <c r="F11" s="17" t="inlineStr">
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>42708915590028</t>
         </is>
       </c>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="G12" s="17" t="inlineStr">
         <is>
           <t>+998 88 803-91-93 / +998 88 726-14-12 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>26-03</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>A.Asraliyev</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Mustafayeva Madina Ortiq qizi</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>AE4846447</t>
         </is>
       </c>
-      <c r="F12" s="14" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
         <is>
           <t>63110085680103</t>
         </is>
       </c>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>26-03</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>A.Asraliyev</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>Primova Husnora Shovkat qizi</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>AC 0443770</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>61310015590029</t>
         </is>
       </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="G14" s="17" t="inlineStr">
         <is>
           <t>+998 87 392-00-25 / +998 87 392-00-21 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>26-03</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>A.Asraliyev</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>Salayeva Dilroz Muroulla qizi</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>AE3039330</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
+      <c r="F15" s="14" t="inlineStr">
         <is>
           <t>60408085730030</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="17" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>26-03</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>A.Asraliyev</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>Umirova Sevinch Avlayor qizi</t>
-        </is>
-      </c>
-      <c r="E15" s="17" t="inlineStr">
-        <is>
-          <t>AD1671106</t>
-        </is>
-      </c>
-      <c r="F15" s="17" t="inlineStr">
-        <is>
-          <t>60906055720101</t>
-        </is>
-      </c>
-      <c r="G15" s="17" t="inlineStr">
-        <is>
-          <t>+998 87 561-52-96 / +998 77 232-28-78 (Otasi / Onasi)</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
@@ -1486,25 +1488,25 @@
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Xurramova Sabina Yuldosh qizi</t>
+          <t>Umirova Sevinch Avlayor qizi</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>AC3081523</t>
+          <t>AD1671106</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>60803048230011</t>
+          <t>60906055720101</t>
         </is>
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>+998 97 960-25-35 / +998 91 216-23-04 (Otasi / Onasi)</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
+          <t>+998 87 561-52-96 / +998 77 232-28-78 (Otasi / Onasi)</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -1517,35 +1519,35 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>26-04</t>
+          <t>26-03</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Xamdamova.M</t>
+          <t>A.Asraliyev</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>G'aniyeva Asila G'ani qizi</t>
+          <t>Xurramova Sabina Yuldosh qizi</t>
         </is>
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>AE5575300</t>
+          <t>AC3081523</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>41011925590038</t>
+          <t>60803048230011</t>
         </is>
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>+998 99 153-48-38 / +998 70 034-22-44 (Otasi / Onasi)</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
+          <t>+998 97 960-25-35 / +998 91 216-23-04 (Otasi / Onasi)</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -1568,25 +1570,25 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Tuychiyeva Farzona Dalerovna</t>
+          <t>G'aniyeva Asila G'ani qizi</t>
         </is>
       </c>
       <c r="E18" s="17" t="inlineStr">
         <is>
-          <t>AE4114421</t>
+          <t>AE5575300</t>
         </is>
       </c>
       <c r="F18" s="17" t="inlineStr">
         <is>
-          <t>60508095680049</t>
+          <t>41011925590038</t>
         </is>
       </c>
       <c r="G18" s="17" t="inlineStr">
         <is>
-          <t>+998 97 573-22-92</t>
-        </is>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
+          <t>+998 99 153-48-38 / +998 70 034-22-44 (Otasi / Onasi)</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -1599,35 +1601,35 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>26-05</t>
+          <t>26-04</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Rayimova.X</t>
+          <t>Xamdamova.M</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Ashirova Gulsanam Abduvali qizi</t>
+          <t>Tuychiyeva Farzona Dalerovna</t>
         </is>
       </c>
       <c r="E19" s="17" t="inlineStr">
         <is>
-          <t>AD6820021</t>
+          <t>AE4114421</t>
         </is>
       </c>
       <c r="F19" s="17" t="inlineStr">
         <is>
-          <t>62311065590082</t>
+          <t>60508095680049</t>
         </is>
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
-          <t>+998 87 636-07-08 / +998 97 636-37-74 (Otasi / Onasi)</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
+          <t>+998 97 573-22-92</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -1650,109 +1652,109 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
+          <t>Ashirova Gulsanam Abduvali qizi</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>AD6820021</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>62311065590082</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>+998 87 636-07-08 / +998 97 636-37-74 (Otasi / Onasi)</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Telefoni bor (bog'lanish mumkin)</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>26-05</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Rayimova.X</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
           <t>Eshboboyeva Fotima Nurali qizi</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>AD0697178</t>
         </is>
       </c>
-      <c r="F20" s="17" t="inlineStr">
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>61306045630044</t>
         </is>
       </c>
-      <c r="G20" s="17" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>+998 88 100-95-04 / +998 97 632-55-74 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H20" s="10" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="14" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>26-05</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>Rayimova.X</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Oripova Sevinch G'olib qizi</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>AE3333890</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F22" s="14" t="inlineStr">
         <is>
           <t>62007085680095</t>
         </is>
       </c>
-      <c r="G21" s="14" t="inlineStr">
+      <c r="G22" s="14" t="inlineStr">
         <is>
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="H22" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="17" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>26-06</t>
-        </is>
-      </c>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>Yuldashev.O</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>Karimova Nozliya Rustamovna</t>
-        </is>
-      </c>
-      <c r="E22" s="17" t="inlineStr">
-        <is>
-          <t>AE4674508</t>
-        </is>
-      </c>
-      <c r="F22" s="17" t="inlineStr">
-        <is>
-          <t>61502085680047</t>
-        </is>
-      </c>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>+998 70 034-95-05 / +998 99 468-84-06 (Otasi / Onasi)</t>
-        </is>
-      </c>
-      <c r="H22" s="10" t="inlineStr">
-        <is>
-          <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
@@ -1773,25 +1775,25 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Mahmatqulova Nilufar Qayum qizi</t>
+          <t>Karimova Nozliya Rustamovna</t>
         </is>
       </c>
       <c r="E23" s="17" t="inlineStr">
         <is>
-          <t>AE6047826</t>
+          <t>AE4674508</t>
         </is>
       </c>
       <c r="F23" s="17" t="inlineStr">
         <is>
-          <t>60806085590115</t>
+          <t>61502085680047</t>
         </is>
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
-          <t>+998 88 384-85-45</t>
-        </is>
-      </c>
-      <c r="H23" s="10" t="inlineStr">
+          <t>+998 70 034-95-05 / +998 99 468-84-06 (Otasi / Onasi)</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -1814,112 +1816,194 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
+          <t>Mahmatqulova Nilufar Qayum qizi</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>AE6047826</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>60806085590115</t>
+        </is>
+      </c>
+      <c r="G24" s="17" t="inlineStr">
+        <is>
+          <t>+998 88 384-85-45</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Telefoni bor (bog'lanish mumkin)</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>26-06</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Yuldashev.O</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
           <t>Mustafayeva Nargiza Ulug'bek qizi</t>
         </is>
       </c>
-      <c r="E24" s="17" t="inlineStr">
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>AB8521319</t>
         </is>
       </c>
-      <c r="F24" s="17" t="inlineStr">
+      <c r="F25" s="17" t="inlineStr">
         <is>
           <t>62906005590060</t>
         </is>
       </c>
-      <c r="G24" s="17" t="inlineStr">
+      <c r="G25" s="17" t="inlineStr">
         <is>
           <t>+998 88 399-00-96</t>
         </is>
       </c>
-      <c r="H24" s="10" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="14" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>26-06</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>Yuldashev.O</t>
         </is>
       </c>
-      <c r="D25" s="16" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
         <is>
           <t>Narziyeva Intizor Iskandar qizi</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>AB5359926</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>40211995680023</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
+      <c r="G26" s="14" t="inlineStr">
         <is>
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="17" t="n">
-        <v>22</v>
-      </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
         <is>
           <t>26-06</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C27" s="18" t="inlineStr">
         <is>
           <t>Yuldashev.O</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D27" s="19" t="inlineStr">
         <is>
           <t>Usmonova Gulnoza Xamdam qizi</t>
         </is>
       </c>
-      <c r="E26" s="17" t="inlineStr">
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>AB5702170</t>
         </is>
       </c>
-      <c r="F26" s="17" t="inlineStr">
+      <c r="F27" s="17" t="inlineStr">
         <is>
           <t>42601925680010</t>
         </is>
       </c>
-      <c r="G26" s="17" t="inlineStr">
+      <c r="G27" s="17" t="inlineStr">
         <is>
           <t>+998 97 066-26-92</t>
         </is>
       </c>
-      <c r="H26" s="10" t="inlineStr">
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr"/>
+      <c r="I27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>26-07</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>Asraliyev.A</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Ergasheva Madina Tulqin qizi</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>AC0429133</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>62501027890026</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>Mavjud emas</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>Telefoni yo'q (aniqlash zarur)</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1927,6 +2011,134 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="79" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>26-01 GURUHI — SO'ROVNOMA TOPSHIRMAGANLAR (1 NAFAR) • Rahbar: Mirzayeva.D</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Guruh rahbarlari tomonidan ma'lumotlarni yig'ish va to'ldirish uchun hisobot</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>T/R</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Guruh</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Guruh rahbari</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Familiya Ism Sharif</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Pasport seriya №</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>JSHSHIR (PINFL)</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>Mavjud telefoni</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>Holati</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>Guruh rahbari qaydi / Yangi telefon / Manzil</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Mirzayeva.D</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Shermatova Gulsun Xurshid qizi</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>AE5836574</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>60802085590029</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>Mavjud emas</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Telefoni yo'q (aniqlash zarur)</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2009,42 +2221,42 @@
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="14" t="n">
+      <c r="A5" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>26-02</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Ochilov.D</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>Nurillayeva Dilsuz Mashrabovna</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>AD4774693</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>42506912640010</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>Mavjud emas</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>Telefoni yo'q (aniqlash zarur)</t>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>Qulmatova Shabbona Azamat qizi</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>AE4905104</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>61008085680019</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>+998 77 833-82-72</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -2065,25 +2277,25 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Qulmatova Shabbona Azamat qizi</t>
+          <t>Samatova Oydin Sulaymon qizi</t>
         </is>
       </c>
       <c r="E6" s="17" t="inlineStr">
         <is>
-          <t>AE4905104</t>
+          <t>AD8980430</t>
         </is>
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>61008085680019</t>
+          <t>42910905720012</t>
         </is>
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>+998 77 833-82-72</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
+          <t>+998 91 219-20-99</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2091,42 +2303,42 @@
       <c r="I6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>26-02</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Ochilov.D</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
-        <is>
-          <t>Samatova Oydin Sulaymon qizi</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>AD8980430</t>
-        </is>
-      </c>
-      <c r="F7" s="17" t="inlineStr">
-        <is>
-          <t>42910905720012</t>
-        </is>
-      </c>
-      <c r="G7" s="17" t="inlineStr">
-        <is>
-          <t>+998 91 219-20-99</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>Telefoni bor (bog'lanish mumkin)</t>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Nurillayeva Dilsuz Mashrabovna</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>AD4774693</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>42506912640010</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Mavjud emas</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Telefoni yo'q (aniqlash zarur)</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
@@ -2136,7 +2348,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2252,7 +2464,7 @@
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
         </is>
@@ -2293,7 +2505,7 @@
           <t>+998 95 259-06-25 / +998 99 152-33-71 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2334,7 +2546,7 @@
           <t>+998 87 358-87-97 / +998 88 632-19-72 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2375,7 +2587,7 @@
           <t>+998 88 803-91-93 / +998 88 726-14-12 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2416,7 +2628,7 @@
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
         </is>
@@ -2457,7 +2669,7 @@
           <t>+998 87 392-00-25 / +998 87 392-00-21 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2498,7 +2710,7 @@
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr">
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
         </is>
@@ -2539,7 +2751,7 @@
           <t>+998 87 561-52-96 / +998 77 232-28-78 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2580,7 +2792,7 @@
           <t>+998 97 960-25-35 / +998 91 216-23-04 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2592,7 +2804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2708,7 +2920,7 @@
           <t>+998 99 153-48-38 / +998 70 034-22-44 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2749,7 +2961,7 @@
           <t>+998 97 573-22-92</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2761,7 +2973,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2877,7 +3089,7 @@
           <t>+998 87 636-07-08 / +998 97 636-37-74 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2918,7 +3130,7 @@
           <t>+998 88 100-95-04 / +998 97 632-55-74 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -2959,7 +3171,7 @@
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
         </is>
@@ -2971,7 +3183,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3087,7 +3299,7 @@
           <t>+998 70 034-95-05 / +998 99 468-84-06 (Otasi / Onasi)</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -3128,7 +3340,7 @@
           <t>+998 88 384-85-45</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -3169,7 +3381,7 @@
           <t>+998 88 399-00-96</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
@@ -3210,7 +3422,7 @@
           <t>Mavjud emas</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>Telefoni yo'q (aniqlash zarur)</t>
         </is>
@@ -3251,12 +3463,140 @@
           <t>+998 97 066-26-92</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>Telefoni bor (bog'lanish mumkin)</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="79" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>26-07 GURUHI — SO'ROVNOMA TOPSHIRMAGANLAR (1 NAFAR) • Rahbar: Asraliyev.A</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Guruh rahbarlari tomonidan ma'lumotlarni yig'ish va to'ldirish uchun hisobot</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>T/R</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Guruh</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Guruh rahbari</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Familiya Ism Sharif</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Pasport seriya №</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>JSHSHIR (PINFL)</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>Mavjud telefoni</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>Holati</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>Guruh rahbari qaydi / Yangi telefon / Manzil</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>26-07</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Asraliyev.A</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Ergasheva Madina Tulqin qizi</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>AC0429133</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>62501027890026</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>Mavjud emas</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Telefoni yo'q (aniqlash zarur)</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>